<commit_message>
v2.0 Complete Release - Security & UX Improvements
Major Features:
- Percentage-based OCR scaling for any resolution
- Live overlay with Pokeball league icons
- SQLite database for tracking in addition to excel
- Complete installer system with auto-start

Security:
- Removed hardcoded API key from testing files
- All sensitive files excluded from repository

UX Improvements:
- Silent OCR mode to eliminate console spam
- 4-second delay after menu detection for rank population
- Database updates for instant overlay refresh
-OCR menu validation (requires all 3 elements)
- Clean console output without source tags

Bug Fixes:
- Fixed Elo comparison logic (higher = better)
- Fixed pandas pyarrow deprecation warning
- Fixed canvas scrollbar coordinate offset
- Fixed KeyError in region display functions
- Fixed overlay not updating rank immediately
</commit_message>
<xml_diff>
--- a/TCGExampleSheet.xlsx
+++ b/TCGExampleSheet.xlsx
@@ -11,6 +11,11 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ExampleDeck" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gholdengo Dragapult" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gholdengo" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet2" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet3" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dengo Pult ATL NEW ED" sheetId="10" state="visible" r:id="rId10"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
@@ -3728,6 +3733,102 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Result</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Opponent Deck</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Rank</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Source</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Win</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Terapagos Noctowl</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>99</v>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>OCR</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Win</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Terapagos Noctowl</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>99</v>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>OCR</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Win</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>99</v>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>OCR</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
@@ -4896,7 +4997,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="A1:A63" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" type="list">
+    <dataValidation sqref="A1:A63" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="0" type="list">
       <formula1>"Win,Loss,Tie"</formula1>
     </dataValidation>
   </dataValidations>
@@ -4910,11 +5011,9 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B1"/>
+  <dimension ref="A1:A1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1"/>
-  </sheetData>
+  <sheetData/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -4925,7 +5024,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B1"/>
+  <dimension ref="A1:B3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4940,6 +5039,139 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Win</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Win</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Dragapult Dusknoir</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:A1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Win</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Poison Archaludon</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Win</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Loss</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Charizard Pidgeot</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Win</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Gholdengo</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:A1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:A1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Loss</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Release v2.1.0: Production-Ready with Professional Installer
Major Features:

- Professional installer with auto-detection and setup

- Headless mode by default (no console window)

- Optional OpenAI API key during installation

- Enhanced Stats Dashboard with battle management

- Process management and console control

- AutoClicker module for automation

New Files:

- INSTALL_COMPLETE_v2.1.bat - Professional installer

- StatsUI.py - Enhanced stats dashboard

- Run_Headless.py/bat - Headless launcher

- AutoClicker.py - Button automation system

- SetupAutoClicker.py - Template capture tool

Improvements:

- Cleaned repository (removed 30+ test/debug files)

- Better error handling and user feedback

- Improved database integration

- Modern UI with glass-morphism design

- Comprehensive documentation

Bug Fixes:

- Fixed rank update issues

- Improved console detection

- Better graph rendering
</commit_message>
<xml_diff>
--- a/TCGExampleSheet.xlsx
+++ b/TCGExampleSheet.xlsx
@@ -16,6 +16,9 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet2" sheetId="8" state="visible" r:id="rId8"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet3" sheetId="9" state="visible" r:id="rId9"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dengo Pult ATL NEW ED" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet4" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet5" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dragapult Dusknoir" sheetId="13" state="visible" r:id="rId13"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
@@ -3829,6 +3832,142 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:A1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:A1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B8"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Win</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Win</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Win</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Win</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Win</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Loss</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Gholdengo</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Loss</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Gholdengo</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Loss</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Gholdengo</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
@@ -5024,7 +5163,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B3"/>
+  <dimension ref="A1:B7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5058,6 +5197,54 @@
         </is>
       </c>
       <c r="B3" t="inlineStr">
+        <is>
+          <t>Dragapult Dusknoir</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Win</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Flareon Noctowl</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Win</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Flareon Noctowl</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Win</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Dragapult Dusknoir</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Win</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
         <is>
           <t>Dragapult Dusknoir</t>
         </is>

</xml_diff>